<commit_message>
More tweaks to validation
</commit_message>
<xml_diff>
--- a/data/data-issues.xlsx
+++ b/data/data-issues.xlsx
@@ -16592,7 +16592,9 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>latitude has values outside valid range (-90 to 90) for: "22-TNV09-02", "22-IIJ07-02", "23-FLS08-04", …, "23-VRD07-01", and "23-XJO04-02".</t>
+          <t>latitude must be within -90 to 90.
+Affected samples:
+"22-TNV09-02", "22-IIJ07-02", "23-FLS08-04", …, "23-VRD07-01", and "23-XJO04-02"</t>
         </is>
       </c>
     </row>
@@ -16604,7 +16606,9 @@
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>longitude has values outside valid range (-180 to 180) for: "22-FKH06-08" and "22-OWZ06-02".</t>
+          <t>longitude must be within -180 to 180.
+Affected samples:
+"22-FKH06-08" and "22-OWZ06-02"</t>
         </is>
       </c>
     </row>
@@ -16616,7 +16620,9 @@
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>Incomplete coordinate pair (one of latitude or longitude is missing) for: "22-YYF05-02" and "22-OIO04-05".</t>
+          <t>Incomplete coordinate pair (one of latitude or longitude is missing).
+Affected samples:
+"22-YYF05-02" and "22-OIO04-05"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove output arg since validation functions return raw issues to be later formatted
</commit_message>
<xml_diff>
--- a/data/data-issues.xlsx
+++ b/data/data-issues.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\soils\tests\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89E2C21-3F2A-4885-83A5-3F4D552BFDA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AFB1B0D-AF4A-4670-8696-BD164EA67AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2538,7 +2538,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2620,8 +2620,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2633,8 +2640,13 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -2696,20 +2708,6 @@
         <color rgb="FF000000"/>
       </left>
       <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thin"/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -2724,13 +2722,14 @@
       </bottom>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf applyAlignment="0" applyBorder="0" applyFill="1" applyFont="1" applyNumberFormat="0" applyProtection="0" fillId="2" fontId="11"/>
+    <xf applyAlignment="0" applyBorder="0" applyFill="1" applyFont="1" applyNumberFormat="0" applyProtection="0" fillId="3" fontId="12"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -2773,15 +2772,21 @@
     <xf applyBorder="1" borderId="5" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
     <xf applyBorder="1" borderId="6" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
     <xf applyBorder="1" borderId="7" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
-    <xf applyBorder="1" borderId="8" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
-    <xf applyBorder="1" borderId="9" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
+    <xf borderId="0" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="4" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="5" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="6" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="7" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
     <xf applyBorder="1" borderId="4" fillId="2" fontId="11" numFmtId="0" xfId="3">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyBorder="1" borderId="6" fillId="2" fontId="11" numFmtId="0" xfId="3">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf applyBorder="1" borderId="8" fillId="2" fontId="11" numFmtId="0" xfId="3">
+    <xf applyBorder="1" borderId="4" fillId="3" fontId="12" numFmtId="0" xfId="4">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="6" fillId="3" fontId="12" numFmtId="0" xfId="4">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyBorder="1" borderId="5" fillId="2" fontId="11" numFmtId="0" xfId="3">
@@ -2790,15 +2795,19 @@
     <xf applyBorder="1" borderId="7" fillId="2" fontId="11" numFmtId="0" xfId="3">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf applyBorder="1" borderId="9" fillId="2" fontId="11" numFmtId="0" xfId="3">
+    <xf applyBorder="1" borderId="5" fillId="3" fontId="12" numFmtId="0" xfId="4">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="7" fillId="3" fontId="12" numFmtId="0" xfId="4">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{CDD386B2-9C7B-4451-A208-3982823DA7A1}"/>
     <cellStyle name="Normal 2 2" xfId="2" xr:uid="{CF77DDE4-DEBD-467F-927F-6AADE9C385D4}"/>
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="4" builtinId="28"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -3569,7 +3578,7 @@
         <v>41</v>
       </c>
       <c r="K2" s="1">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="L2" s="1">
         <v>36</v>
@@ -3926,7 +3935,7 @@
         <v>72</v>
       </c>
       <c r="H5" s="1">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="I5" s="1">
         <v>-123</v>
@@ -4059,9 +4068,6 @@
       <c r="K6" s="1">
         <v>28</v>
       </c>
-      <c r="L6" s="1">
-        <v>43</v>
-      </c>
       <c r="M6" s="1">
         <v>29</v>
       </c>
@@ -4170,7 +4176,7 @@
         <v>88</v>
       </c>
       <c r="H7" s="1">
-        <v>-150</v>
+        <v>47</v>
       </c>
       <c r="I7" s="1">
         <v>-120</v>
@@ -4426,7 +4432,7 @@
         <v>71</v>
       </c>
       <c r="L9" s="1">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="M9" s="1">
         <v>2</v>
@@ -4538,6 +4544,9 @@
       <c r="G10" s="1" t="s">
         <v>80</v>
       </c>
+      <c r="H10" s="1">
+        <v>47</v>
+      </c>
       <c r="I10" s="1">
         <v>-119</v>
       </c>
@@ -4660,14 +4669,11 @@
       <c r="H11" s="1">
         <v>47</v>
       </c>
+      <c r="I11" s="1">
+        <v>-119</v>
+      </c>
       <c r="J11" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="K11" s="1">
-        <v>53</v>
-      </c>
-      <c r="L11" s="1">
-        <v>41</v>
       </c>
       <c r="M11" s="1">
         <v>6</v>
@@ -4780,7 +4786,7 @@
         <v>48</v>
       </c>
       <c r="I12" s="1">
-        <v>-200</v>
+        <v>-123</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>62</v>
@@ -5148,15 +5154,6 @@
       <c r="J15" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K15" s="1">
-        <v>61</v>
-      </c>
-      <c r="L15" s="1">
-        <v>33</v>
-      </c>
-      <c r="M15" s="1">
-        <v>6</v>
-      </c>
       <c r="N15" s="1">
         <v>0.55000000000000004</v>
       </c>
@@ -5625,16 +5622,7 @@
         <v>47</v>
       </c>
       <c r="I19" s="1">
-        <v>250</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="K19" s="1">
-        <v>19</v>
-      </c>
-      <c r="L19" s="1">
-        <v>53</v>
+        <v>-123</v>
       </c>
       <c r="M19" s="1">
         <v>28</v>
@@ -5871,17 +5859,11 @@
       <c r="I21" s="1">
         <v>-123</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="K21" s="1">
         <v>42</v>
       </c>
       <c r="L21" s="1">
         <v>48</v>
-      </c>
-      <c r="M21" s="1">
-        <v>10</v>
       </c>
       <c r="N21" s="1">
         <v>1.1000000000000001</v>
@@ -6243,11 +6225,8 @@
       <c r="K24" s="1">
         <v>44</v>
       </c>
-      <c r="L24" s="1">
-        <v>42</v>
-      </c>
       <c r="M24" s="1">
-        <v>14</v>
+        <v>400</v>
       </c>
       <c r="N24" s="1">
         <v>1.18</v>
@@ -9904,7 +9883,7 @@
         <v>55</v>
       </c>
       <c r="H54" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I54" s="1">
         <v>-117</v>
@@ -10026,7 +10005,7 @@
         <v>55</v>
       </c>
       <c r="H55" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I55" s="1">
         <v>-117</v>
@@ -10148,7 +10127,7 @@
         <v>55</v>
       </c>
       <c r="H56" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I56" s="1">
         <v>-117</v>
@@ -10270,7 +10249,7 @@
         <v>58</v>
       </c>
       <c r="H57" s="1">
-        <v>200</v>
+        <v>46</v>
       </c>
       <c r="I57" s="1">
         <v>-123</v>
@@ -10392,7 +10371,7 @@
         <v>53</v>
       </c>
       <c r="H58" s="1">
-        <v>200</v>
+        <v>46</v>
       </c>
       <c r="I58" s="1">
         <v>-123</v>
@@ -10514,7 +10493,7 @@
         <v>40</v>
       </c>
       <c r="H59" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I59" s="1">
         <v>-119</v>
@@ -10636,7 +10615,7 @@
         <v>40</v>
       </c>
       <c r="H60" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I60" s="1">
         <v>-121</v>
@@ -10758,7 +10737,7 @@
         <v>68</v>
       </c>
       <c r="H61" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I61" s="1">
         <v>-123</v>
@@ -10880,7 +10859,7 @@
         <v>55</v>
       </c>
       <c r="H62" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I62" s="1">
         <v>-118</v>
@@ -11002,7 +10981,7 @@
         <v>80</v>
       </c>
       <c r="H63" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I63" s="1">
         <v>-120</v>
@@ -11127,7 +11106,7 @@
         <v>53</v>
       </c>
       <c r="H64" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I64" s="1">
         <v>-120</v>
@@ -11252,7 +11231,7 @@
         <v>53</v>
       </c>
       <c r="H65" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I65" s="1">
         <v>-117</v>
@@ -11374,7 +11353,7 @@
         <v>53</v>
       </c>
       <c r="H66" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I66" s="1">
         <v>-117</v>
@@ -11496,7 +11475,7 @@
         <v>47</v>
       </c>
       <c r="H67" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I67" s="1">
         <v>-122</v>
@@ -11618,7 +11597,7 @@
         <v>47</v>
       </c>
       <c r="H68" s="1">
-        <v>200</v>
+        <v>49</v>
       </c>
       <c r="I68" s="1">
         <v>-123</v>
@@ -11740,7 +11719,7 @@
         <v>78</v>
       </c>
       <c r="H69" s="1">
-        <v>200</v>
+        <v>49</v>
       </c>
       <c r="I69" s="1">
         <v>-123</v>
@@ -11862,7 +11841,7 @@
         <v>80</v>
       </c>
       <c r="H70" s="1">
-        <v>200</v>
+        <v>46</v>
       </c>
       <c r="I70" s="1">
         <v>-118</v>
@@ -11984,7 +11963,7 @@
         <v>72</v>
       </c>
       <c r="H71" s="1">
-        <v>200</v>
+        <v>49</v>
       </c>
       <c r="I71" s="1">
         <v>-122</v>
@@ -16549,7 +16528,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
@@ -16585,44 +16564,58 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>latitude must be within -90 to 90.
+          <t>Texture fractions must be between 0 and 100.
 Affected samples:
-"22-TNV09-02", "22-IIJ07-02", "23-FLS08-04", …, "23-VRD07-01", and "23-XJO04-02"</t>
+"22-OSN03-01" and "22-XTO07-03"</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
-          <t>longitude must be within -180 to 180.
+          <t>Texture fractions must sum to 100 (+/- 1).
 Affected samples:
-"22-FKH06-08" and "22-OWZ06-02"</t>
+"22-OSN03-01" and "22-UGU06-02"</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>warning</t>
         </is>
       </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>Incomplete coordinate pair (one of latitude or longitude is missing).
+          <t>At least two texture fractions must be provided to classify texture class.
 Affected samples:
-"22-YYF05-02" and "22-OIO04-05"</t>
+"22-OWZ06-02"</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t>One texture fraction is missing and will be computed as 100 minus the other two.
+Affected samples:
+"22-YIC08-01", "22-YGV09-02", and "22-XTO07-03"</t>
         </is>
       </c>
     </row>

</xml_diff>